<commit_message>
Updated ESP_grids model - 2025-09-23 00:01
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
+++ b/VerveStacks_ESP_grids/SubRES_Tmpl/SubRES_New_RE_and_Conventional_Trans.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ESP_grids\SubRES_Tmpl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6A60E7D-075D-43A8-8414-FF271D1FCBDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A7B49FF-08CC-4811-8580-B6681568969A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1200" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1320" uniqueCount="359">
   <si>
     <t>PSET_PN</t>
   </si>
@@ -310,6 +310,12 @@
     <t>at grid node - ES210-400</t>
   </si>
   <si>
+    <t>w190110739-400</t>
+  </si>
+  <si>
+    <t>at grid node - w190110739-400</t>
+  </si>
+  <si>
     <t>ES251-400</t>
   </si>
   <si>
@@ -502,12 +508,6 @@
     <t>at grid node - w140011919-400</t>
   </si>
   <si>
-    <t>w190110739-400</t>
-  </si>
-  <si>
-    <t>at grid node - w190110739-400</t>
-  </si>
-  <si>
     <t>w51822825-400</t>
   </si>
   <si>
@@ -523,6 +523,12 @@
     <t>at grid node - w143483666-400</t>
   </si>
   <si>
+    <t>w51188420-400</t>
+  </si>
+  <si>
+    <t>at grid node - w51188420-400</t>
+  </si>
+  <si>
     <t>w47911346-400</t>
   </si>
   <si>
@@ -649,12 +655,6 @@
     <t>at grid node - w487381592-400</t>
   </si>
   <si>
-    <t>w51188420-400</t>
-  </si>
-  <si>
-    <t>at grid node - w51188420-400</t>
-  </si>
-  <si>
     <t>ES396-400</t>
   </si>
   <si>
@@ -691,6 +691,12 @@
     <t>at grid node - w189184531-400</t>
   </si>
   <si>
+    <t>w58928252-400</t>
+  </si>
+  <si>
+    <t>at grid node - w58928252-400</t>
+  </si>
+  <si>
     <t>ES26-400</t>
   </si>
   <si>
@@ -784,18 +790,120 @@
     <t>at grid node - w169999915-400</t>
   </si>
   <si>
+    <t>w86512030-400</t>
+  </si>
+  <si>
+    <t>at grid node - w86512030-400</t>
+  </si>
+  <si>
     <t>w1120397197-400</t>
   </si>
   <si>
     <t>at grid node - w1120397197-400</t>
   </si>
   <si>
+    <t>w340399370-400</t>
+  </si>
+  <si>
+    <t>at grid node - w340399370-400</t>
+  </si>
+  <si>
+    <t>w145823172-400</t>
+  </si>
+  <si>
+    <t>at grid node - w145823172-400</t>
+  </si>
+  <si>
+    <t>w97199647-400</t>
+  </si>
+  <si>
+    <t>at grid node - w97199647-400</t>
+  </si>
+  <si>
+    <t>ES1-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES1-400</t>
+  </si>
+  <si>
+    <t>w144941889-400</t>
+  </si>
+  <si>
+    <t>at grid node - w144941889-400</t>
+  </si>
+  <si>
+    <t>w170954487-400</t>
+  </si>
+  <si>
+    <t>at grid node - w170954487-400</t>
+  </si>
+  <si>
+    <t>w772400244-400</t>
+  </si>
+  <si>
+    <t>at grid node - w772400244-400</t>
+  </si>
+  <si>
+    <t>w170485453-400</t>
+  </si>
+  <si>
+    <t>at grid node - w170485453-400</t>
+  </si>
+  <si>
+    <t>ES376-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES376-400</t>
+  </si>
+  <si>
+    <t>w260018670-400</t>
+  </si>
+  <si>
+    <t>at grid node - w260018670-400</t>
+  </si>
+  <si>
+    <t>w1032009205-400</t>
+  </si>
+  <si>
+    <t>at grid node - w1032009205-400</t>
+  </si>
+  <si>
     <t>w651711449-400</t>
   </si>
   <si>
     <t>at grid node - w651711449-400</t>
   </si>
   <si>
+    <t>ES339-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES339-400</t>
+  </si>
+  <si>
+    <t>w1246115410-400</t>
+  </si>
+  <si>
+    <t>at grid node - w1246115410-400</t>
+  </si>
+  <si>
+    <t>w144787749-400</t>
+  </si>
+  <si>
+    <t>at grid node - w144787749-400</t>
+  </si>
+  <si>
+    <t>w27936937-400</t>
+  </si>
+  <si>
+    <t>at grid node - w27936937-400</t>
+  </si>
+  <si>
+    <t>w283348372-400</t>
+  </si>
+  <si>
+    <t>at grid node - w283348372-400</t>
+  </si>
+  <si>
     <t>w1054312727-400</t>
   </si>
   <si>
@@ -808,34 +916,58 @@
     <t>at grid node - w986410945-400</t>
   </si>
   <si>
-    <t>w1246115410-400</t>
-  </si>
-  <si>
-    <t>at grid node - w1246115410-400</t>
-  </si>
-  <si>
-    <t>w1032009205-400</t>
-  </si>
-  <si>
-    <t>at grid node - w1032009205-400</t>
-  </si>
-  <si>
     <t>w28683005-400</t>
   </si>
   <si>
     <t>at grid node - w28683005-400</t>
   </si>
   <si>
+    <t>w677413570-400</t>
+  </si>
+  <si>
+    <t>at grid node - w677413570-400</t>
+  </si>
+  <si>
+    <t>w931181199-400</t>
+  </si>
+  <si>
+    <t>at grid node - w931181199-400</t>
+  </si>
+  <si>
+    <t>w190236352-400</t>
+  </si>
+  <si>
+    <t>at grid node - w190236352-400</t>
+  </si>
+  <si>
+    <t>w189577215-400</t>
+  </si>
+  <si>
+    <t>at grid node - w189577215-400</t>
+  </si>
+  <si>
     <t>w144909709-400</t>
   </si>
   <si>
     <t>at grid node - w144909709-400</t>
   </si>
   <si>
-    <t>ES339-400</t>
-  </si>
-  <si>
-    <t>at grid node - ES339-400</t>
+    <t>w118057369-400</t>
+  </si>
+  <si>
+    <t>at grid node - w118057369-400</t>
+  </si>
+  <si>
+    <t>w1267694217-400</t>
+  </si>
+  <si>
+    <t>at grid node - w1267694217-400</t>
+  </si>
+  <si>
+    <t>w683693772-400</t>
+  </si>
+  <si>
+    <t>at grid node - w683693772-400</t>
   </si>
   <si>
     <t>w788716327-400</t>
@@ -844,16 +976,52 @@
     <t>at grid node - w788716327-400</t>
   </si>
   <si>
+    <t>ES119-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES119-400</t>
+  </si>
+  <si>
+    <t>ES139-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES139-400</t>
+  </si>
+  <si>
+    <t>w145461765-400</t>
+  </si>
+  <si>
+    <t>at grid node - w145461765-400</t>
+  </si>
+  <si>
+    <t>w1042227719-400</t>
+  </si>
+  <si>
+    <t>at grid node - w1042227719-400</t>
+  </si>
+  <si>
+    <t>w28308003-400</t>
+  </si>
+  <si>
+    <t>at grid node - w28308003-400</t>
+  </si>
+  <si>
     <t>w327268322-400</t>
   </si>
   <si>
     <t>at grid node - w327268322-400</t>
   </si>
   <si>
-    <t>w118057369-400</t>
-  </si>
-  <si>
-    <t>at grid node - w118057369-400</t>
+    <t>ES174-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES174-400</t>
+  </si>
+  <si>
+    <t>ES264-400</t>
+  </si>
+  <si>
+    <t>at grid node - ES264-400</t>
   </si>
   <si>
     <t>ES302-400</t>
@@ -901,24 +1069,12 @@
     <t>at grid node - w129441519-400</t>
   </si>
   <si>
-    <t>w144787749-400</t>
-  </si>
-  <si>
-    <t>at grid node - w144787749-400</t>
-  </si>
-  <si>
     <t>w1252094933-400</t>
   </si>
   <si>
     <t>at grid node - w1252094933-400</t>
   </si>
   <si>
-    <t>w170954487-400</t>
-  </si>
-  <si>
-    <t>at grid node - w170954487-400</t>
-  </si>
-  <si>
     <t>w171251565-400</t>
   </si>
   <si>
@@ -931,22 +1087,10 @@
     <t>at grid node - w729485840-400</t>
   </si>
   <si>
-    <t>w772400244-400</t>
-  </si>
-  <si>
-    <t>at grid node - w772400244-400</t>
-  </si>
-  <si>
     <t>w71796402-400</t>
   </si>
   <si>
     <t>at grid node - w71796402-400</t>
-  </si>
-  <si>
-    <t>ES174-400</t>
-  </si>
-  <si>
-    <t>at grid node - ES174-400</t>
   </si>
   <si>
     <t>ES239-400</t>
@@ -1298,7 +1442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{268E9BAB-B98F-4B82-9042-51EABC9ED525}">
-  <dimension ref="B3:T107"/>
+  <dimension ref="B3:T135"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="3" spans="2:20" x14ac:dyDescent="0.45">
@@ -1421,19 +1565,19 @@
         <v>80</v>
       </c>
       <c r="O11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q11" t="s">
         <v>78</v>
       </c>
       <c r="R11" t="s">
-        <v>276</v>
+        <v>332</v>
       </c>
       <c r="S11" t="s">
-        <v>277</v>
+        <v>333</v>
       </c>
       <c r="T11" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.45">
@@ -1471,19 +1615,19 @@
         <v>83</v>
       </c>
       <c r="O12" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q12" t="s">
         <v>78</v>
       </c>
       <c r="R12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="S12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T12" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" spans="2:20" x14ac:dyDescent="0.45">
@@ -1521,19 +1665,19 @@
         <v>85</v>
       </c>
       <c r="O13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q13" t="s">
         <v>78</v>
       </c>
       <c r="R13" t="s">
-        <v>260</v>
+        <v>292</v>
       </c>
       <c r="S13" t="s">
-        <v>261</v>
+        <v>293</v>
       </c>
       <c r="T13" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="14" spans="2:20" x14ac:dyDescent="0.45">
@@ -1571,19 +1715,19 @@
         <v>87</v>
       </c>
       <c r="O14" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q14" t="s">
         <v>78</v>
       </c>
       <c r="R14" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="S14" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="T14" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="2:20" x14ac:dyDescent="0.45">
@@ -1621,19 +1765,19 @@
         <v>89</v>
       </c>
       <c r="O15" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q15" t="s">
         <v>78</v>
       </c>
       <c r="R15" t="s">
-        <v>279</v>
+        <v>335</v>
       </c>
       <c r="S15" t="s">
-        <v>280</v>
+        <v>336</v>
       </c>
       <c r="T15" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="16" spans="2:20" x14ac:dyDescent="0.45">
@@ -1665,25 +1809,25 @@
         <v>78</v>
       </c>
       <c r="M16" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N16" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="O16" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q16" t="s">
         <v>78</v>
       </c>
       <c r="R16" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="S16" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="T16" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.45">
@@ -1703,10 +1847,10 @@
         <v>78</v>
       </c>
       <c r="H17" t="s">
-        <v>92</v>
+        <v>169</v>
       </c>
       <c r="I17" t="s">
-        <v>93</v>
+        <v>170</v>
       </c>
       <c r="J17" t="s">
         <v>158</v>
@@ -1721,19 +1865,19 @@
         <v>91</v>
       </c>
       <c r="O17" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q17" t="s">
         <v>78</v>
       </c>
       <c r="R17" t="s">
-        <v>281</v>
+        <v>337</v>
       </c>
       <c r="S17" t="s">
-        <v>282</v>
+        <v>338</v>
       </c>
       <c r="T17" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.45">
@@ -1753,10 +1897,10 @@
         <v>78</v>
       </c>
       <c r="H18" t="s">
-        <v>169</v>
+        <v>94</v>
       </c>
       <c r="I18" t="s">
-        <v>170</v>
+        <v>95</v>
       </c>
       <c r="J18" t="s">
         <v>158</v>
@@ -1771,19 +1915,19 @@
         <v>93</v>
       </c>
       <c r="O18" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q18" t="s">
         <v>78</v>
       </c>
       <c r="R18" t="s">
-        <v>283</v>
+        <v>339</v>
       </c>
       <c r="S18" t="s">
-        <v>284</v>
+        <v>340</v>
       </c>
       <c r="T18" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.45">
@@ -1821,19 +1965,19 @@
         <v>95</v>
       </c>
       <c r="O19" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q19" t="s">
         <v>78</v>
       </c>
       <c r="R19" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="S19" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="T19" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.45">
@@ -1871,19 +2015,19 @@
         <v>97</v>
       </c>
       <c r="O20" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q20" t="s">
         <v>78</v>
       </c>
       <c r="R20" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="S20" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="T20" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.45">
@@ -1921,19 +2065,19 @@
         <v>99</v>
       </c>
       <c r="O21" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q21" t="s">
         <v>78</v>
       </c>
       <c r="R21" t="s">
-        <v>285</v>
+        <v>341</v>
       </c>
       <c r="S21" t="s">
-        <v>286</v>
+        <v>342</v>
       </c>
       <c r="T21" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.45">
@@ -1971,19 +2115,19 @@
         <v>101</v>
       </c>
       <c r="O22" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q22" t="s">
         <v>78</v>
       </c>
       <c r="R22" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="S22" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="T22" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.45">
@@ -2003,10 +2147,10 @@
         <v>78</v>
       </c>
       <c r="H23" t="s">
-        <v>90</v>
+        <v>179</v>
       </c>
       <c r="I23" t="s">
-        <v>91</v>
+        <v>180</v>
       </c>
       <c r="J23" t="s">
         <v>158</v>
@@ -2021,19 +2165,19 @@
         <v>103</v>
       </c>
       <c r="O23" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q23" t="s">
         <v>78</v>
       </c>
       <c r="R23" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="S23" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="T23" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.45">
@@ -2053,10 +2197,10 @@
         <v>78</v>
       </c>
       <c r="H24" t="s">
-        <v>179</v>
+        <v>92</v>
       </c>
       <c r="I24" t="s">
-        <v>180</v>
+        <v>93</v>
       </c>
       <c r="J24" t="s">
         <v>158</v>
@@ -2071,19 +2215,19 @@
         <v>105</v>
       </c>
       <c r="O24" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q24" t="s">
         <v>78</v>
       </c>
       <c r="R24" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="S24" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="T24" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="25" spans="2:20" x14ac:dyDescent="0.45">
@@ -2115,25 +2259,25 @@
         <v>78</v>
       </c>
       <c r="M25" t="s">
-        <v>183</v>
+        <v>106</v>
       </c>
       <c r="N25" t="s">
-        <v>184</v>
+        <v>107</v>
       </c>
       <c r="O25" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q25" t="s">
         <v>78</v>
       </c>
       <c r="R25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="S25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="T25" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="26" spans="2:20" x14ac:dyDescent="0.45">
@@ -2165,25 +2309,25 @@
         <v>78</v>
       </c>
       <c r="M26" t="s">
-        <v>106</v>
+        <v>185</v>
       </c>
       <c r="N26" t="s">
-        <v>107</v>
+        <v>186</v>
       </c>
       <c r="O26" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q26" t="s">
         <v>78</v>
       </c>
       <c r="R26" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="S26" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="T26" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.45">
@@ -2221,19 +2365,19 @@
         <v>109</v>
       </c>
       <c r="O27" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q27" t="s">
         <v>78</v>
       </c>
       <c r="R27" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="S27" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="T27" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.45">
@@ -2253,10 +2397,10 @@
         <v>78</v>
       </c>
       <c r="H28" t="s">
-        <v>84</v>
+        <v>187</v>
       </c>
       <c r="I28" t="s">
-        <v>85</v>
+        <v>188</v>
       </c>
       <c r="J28" t="s">
         <v>158</v>
@@ -2271,19 +2415,19 @@
         <v>111</v>
       </c>
       <c r="O28" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q28" t="s">
         <v>78</v>
       </c>
       <c r="R28" t="s">
-        <v>289</v>
+        <v>343</v>
       </c>
       <c r="S28" t="s">
-        <v>290</v>
+        <v>344</v>
       </c>
       <c r="T28" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="29" spans="2:20" x14ac:dyDescent="0.45">
@@ -2303,10 +2447,10 @@
         <v>78</v>
       </c>
       <c r="H29" t="s">
-        <v>187</v>
+        <v>84</v>
       </c>
       <c r="I29" t="s">
-        <v>188</v>
+        <v>85</v>
       </c>
       <c r="J29" t="s">
         <v>158</v>
@@ -2321,19 +2465,19 @@
         <v>113</v>
       </c>
       <c r="O29" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q29" t="s">
         <v>78</v>
       </c>
       <c r="R29" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="S29" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="T29" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="30" spans="2:20" x14ac:dyDescent="0.45">
@@ -2371,19 +2515,19 @@
         <v>115</v>
       </c>
       <c r="O30" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q30" t="s">
         <v>78</v>
       </c>
       <c r="R30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="S30" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="T30" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="31" spans="2:20" x14ac:dyDescent="0.45">
@@ -2421,19 +2565,19 @@
         <v>117</v>
       </c>
       <c r="O31" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q31" t="s">
         <v>78</v>
       </c>
       <c r="R31" t="s">
-        <v>291</v>
+        <v>264</v>
       </c>
       <c r="S31" t="s">
-        <v>292</v>
+        <v>265</v>
       </c>
       <c r="T31" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="32" spans="2:20" x14ac:dyDescent="0.45">
@@ -2465,25 +2609,25 @@
         <v>78</v>
       </c>
       <c r="M32" t="s">
-        <v>205</v>
+        <v>118</v>
       </c>
       <c r="N32" t="s">
-        <v>206</v>
+        <v>119</v>
       </c>
       <c r="O32" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q32" t="s">
         <v>78</v>
       </c>
       <c r="R32" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="S32" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="T32" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="33" spans="2:20" x14ac:dyDescent="0.45">
@@ -2503,10 +2647,10 @@
         <v>78</v>
       </c>
       <c r="H33" t="s">
-        <v>98</v>
+        <v>195</v>
       </c>
       <c r="I33" t="s">
-        <v>99</v>
+        <v>196</v>
       </c>
       <c r="J33" t="s">
         <v>158</v>
@@ -2515,25 +2659,25 @@
         <v>78</v>
       </c>
       <c r="M33" t="s">
-        <v>118</v>
+        <v>205</v>
       </c>
       <c r="N33" t="s">
-        <v>119</v>
+        <v>206</v>
       </c>
       <c r="O33" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q33" t="s">
         <v>78</v>
       </c>
       <c r="R33" t="s">
-        <v>293</v>
+        <v>345</v>
       </c>
       <c r="S33" t="s">
-        <v>294</v>
+        <v>346</v>
       </c>
       <c r="T33" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="34" spans="2:20" x14ac:dyDescent="0.45">
@@ -2553,10 +2697,10 @@
         <v>78</v>
       </c>
       <c r="H34" t="s">
-        <v>195</v>
+        <v>100</v>
       </c>
       <c r="I34" t="s">
-        <v>196</v>
+        <v>101</v>
       </c>
       <c r="J34" t="s">
         <v>158</v>
@@ -2571,19 +2715,19 @@
         <v>121</v>
       </c>
       <c r="O34" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q34" t="s">
         <v>78</v>
       </c>
       <c r="R34" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="S34" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="T34" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="35" spans="2:20" x14ac:dyDescent="0.45">
@@ -2615,25 +2759,25 @@
         <v>78</v>
       </c>
       <c r="M35" t="s">
-        <v>240</v>
+        <v>122</v>
       </c>
       <c r="N35" t="s">
-        <v>241</v>
+        <v>123</v>
       </c>
       <c r="O35" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q35" t="s">
         <v>78</v>
       </c>
       <c r="R35" t="s">
-        <v>154</v>
+        <v>90</v>
       </c>
       <c r="S35" t="s">
-        <v>155</v>
+        <v>91</v>
       </c>
       <c r="T35" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="36" spans="2:20" x14ac:dyDescent="0.45">
@@ -2653,10 +2797,10 @@
         <v>78</v>
       </c>
       <c r="H36" t="s">
-        <v>199</v>
+        <v>82</v>
       </c>
       <c r="I36" t="s">
-        <v>200</v>
+        <v>83</v>
       </c>
       <c r="J36" t="s">
         <v>158</v>
@@ -2665,25 +2809,25 @@
         <v>78</v>
       </c>
       <c r="M36" t="s">
-        <v>122</v>
+        <v>242</v>
       </c>
       <c r="N36" t="s">
-        <v>123</v>
+        <v>243</v>
       </c>
       <c r="O36" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q36" t="s">
         <v>78</v>
       </c>
       <c r="R36" t="s">
-        <v>268</v>
+        <v>322</v>
       </c>
       <c r="S36" t="s">
-        <v>269</v>
+        <v>323</v>
       </c>
       <c r="T36" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="37" spans="2:20" x14ac:dyDescent="0.45">
@@ -2703,10 +2847,10 @@
         <v>78</v>
       </c>
       <c r="H37" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="I37" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="J37" t="s">
         <v>158</v>
@@ -2721,19 +2865,19 @@
         <v>125</v>
       </c>
       <c r="O37" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q37" t="s">
         <v>78</v>
       </c>
       <c r="R37" t="s">
-        <v>295</v>
+        <v>347</v>
       </c>
       <c r="S37" t="s">
-        <v>296</v>
+        <v>348</v>
       </c>
       <c r="T37" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="38" spans="2:20" x14ac:dyDescent="0.45">
@@ -2753,10 +2897,10 @@
         <v>78</v>
       </c>
       <c r="H38" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="I38" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J38" t="s">
         <v>158</v>
@@ -2771,19 +2915,19 @@
         <v>127</v>
       </c>
       <c r="O38" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q38" t="s">
         <v>78</v>
       </c>
       <c r="R38" t="s">
-        <v>297</v>
+        <v>266</v>
       </c>
       <c r="S38" t="s">
-        <v>298</v>
+        <v>267</v>
       </c>
       <c r="T38" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="39" spans="2:20" x14ac:dyDescent="0.45">
@@ -2803,10 +2947,10 @@
         <v>78</v>
       </c>
       <c r="H39" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="I39" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="J39" t="s">
         <v>158</v>
@@ -2821,19 +2965,19 @@
         <v>129</v>
       </c>
       <c r="O39" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q39" t="s">
         <v>78</v>
       </c>
       <c r="R39" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="S39" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="T39" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="40" spans="2:20" x14ac:dyDescent="0.45">
@@ -2853,10 +2997,10 @@
         <v>78</v>
       </c>
       <c r="H40" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="I40" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="J40" t="s">
         <v>158</v>
@@ -2865,25 +3009,25 @@
         <v>78</v>
       </c>
       <c r="M40" t="s">
-        <v>242</v>
+        <v>130</v>
       </c>
       <c r="N40" t="s">
-        <v>243</v>
+        <v>131</v>
       </c>
       <c r="O40" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q40" t="s">
         <v>78</v>
       </c>
       <c r="R40" t="s">
-        <v>299</v>
+        <v>349</v>
       </c>
       <c r="S40" t="s">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="T40" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="41" spans="2:20" x14ac:dyDescent="0.45">
@@ -2903,10 +3047,10 @@
         <v>78</v>
       </c>
       <c r="H41" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="I41" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="J41" t="s">
         <v>158</v>
@@ -2915,25 +3059,25 @@
         <v>78</v>
       </c>
       <c r="M41" t="s">
-        <v>130</v>
+        <v>244</v>
       </c>
       <c r="N41" t="s">
-        <v>131</v>
+        <v>245</v>
       </c>
       <c r="O41" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q41" t="s">
         <v>78</v>
       </c>
       <c r="R41" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="S41" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="T41" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42" spans="2:20" x14ac:dyDescent="0.45">
@@ -2953,10 +3097,10 @@
         <v>78</v>
       </c>
       <c r="H42" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="I42" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="J42" t="s">
         <v>158</v>
@@ -2971,19 +3115,19 @@
         <v>133</v>
       </c>
       <c r="O42" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q42" t="s">
         <v>78</v>
       </c>
       <c r="R42" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="S42" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="T42" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="43" spans="2:20" x14ac:dyDescent="0.45">
@@ -3003,10 +3147,10 @@
         <v>78</v>
       </c>
       <c r="H43" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="I43" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="J43" t="s">
         <v>158</v>
@@ -3015,25 +3159,25 @@
         <v>78</v>
       </c>
       <c r="M43" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="N43" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="O43" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q43" t="s">
         <v>78</v>
       </c>
       <c r="R43" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="S43" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="T43" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.45">
@@ -3053,10 +3197,10 @@
         <v>78</v>
       </c>
       <c r="H44" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="I44" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="J44" t="s">
         <v>158</v>
@@ -3065,25 +3209,25 @@
         <v>78</v>
       </c>
       <c r="M44" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="N44" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="O44" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q44" t="s">
         <v>78</v>
       </c>
       <c r="R44" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="S44" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="T44" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="45" spans="2:20" x14ac:dyDescent="0.45">
@@ -3103,10 +3247,10 @@
         <v>78</v>
       </c>
       <c r="H45" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="I45" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="J45" t="s">
         <v>158</v>
@@ -3121,19 +3265,19 @@
         <v>137</v>
       </c>
       <c r="O45" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q45" t="s">
         <v>78</v>
       </c>
       <c r="R45" t="s">
-        <v>301</v>
+        <v>324</v>
       </c>
       <c r="S45" t="s">
-        <v>302</v>
+        <v>325</v>
       </c>
       <c r="T45" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="46" spans="2:20" x14ac:dyDescent="0.45">
@@ -3153,10 +3297,10 @@
         <v>78</v>
       </c>
       <c r="H46" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="I46" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="J46" t="s">
         <v>158</v>
@@ -3171,19 +3315,19 @@
         <v>139</v>
       </c>
       <c r="O46" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q46" t="s">
         <v>78</v>
       </c>
       <c r="R46" t="s">
-        <v>303</v>
+        <v>351</v>
       </c>
       <c r="S46" t="s">
-        <v>304</v>
+        <v>352</v>
       </c>
       <c r="T46" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="47" spans="2:20" x14ac:dyDescent="0.45">
@@ -3203,10 +3347,10 @@
         <v>78</v>
       </c>
       <c r="H47" t="s">
-        <v>82</v>
+        <v>219</v>
       </c>
       <c r="I47" t="s">
-        <v>83</v>
+        <v>220</v>
       </c>
       <c r="J47" t="s">
         <v>158</v>
@@ -3221,19 +3365,19 @@
         <v>141</v>
       </c>
       <c r="O47" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q47" t="s">
         <v>78</v>
       </c>
       <c r="R47" t="s">
-        <v>305</v>
+        <v>353</v>
       </c>
       <c r="S47" t="s">
-        <v>306</v>
+        <v>354</v>
       </c>
       <c r="T47" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="48" spans="2:20" x14ac:dyDescent="0.45">
@@ -3265,25 +3409,25 @@
         <v>78</v>
       </c>
       <c r="M48" t="s">
-        <v>244</v>
+        <v>142</v>
       </c>
       <c r="N48" t="s">
-        <v>245</v>
+        <v>143</v>
       </c>
       <c r="O48" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q48" t="s">
         <v>78</v>
       </c>
       <c r="R48" t="s">
-        <v>307</v>
+        <v>355</v>
       </c>
       <c r="S48" t="s">
-        <v>308</v>
+        <v>356</v>
       </c>
       <c r="T48" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="49" spans="7:20" x14ac:dyDescent="0.45">
@@ -3303,25 +3447,25 @@
         <v>78</v>
       </c>
       <c r="M49" t="s">
-        <v>144</v>
+        <v>246</v>
       </c>
       <c r="N49" t="s">
-        <v>145</v>
+        <v>247</v>
       </c>
       <c r="O49" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q49" t="s">
         <v>78</v>
       </c>
       <c r="R49" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="S49" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="T49" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="50" spans="7:20" x14ac:dyDescent="0.45">
@@ -3347,19 +3491,19 @@
         <v>147</v>
       </c>
       <c r="O50" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q50" t="s">
         <v>78</v>
       </c>
       <c r="R50" t="s">
-        <v>309</v>
+        <v>357</v>
       </c>
       <c r="S50" t="s">
-        <v>310</v>
+        <v>358</v>
       </c>
       <c r="T50" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="51" spans="7:20" x14ac:dyDescent="0.45">
@@ -3385,7 +3529,7 @@
         <v>149</v>
       </c>
       <c r="O51" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="Q51" t="s">
         <v>78</v>
@@ -3397,7 +3541,7 @@
         <v>210</v>
       </c>
       <c r="T51" t="s">
-        <v>278</v>
+        <v>334</v>
       </c>
     </row>
     <row r="52" spans="7:20" x14ac:dyDescent="0.45">
@@ -3423,7 +3567,7 @@
         <v>151</v>
       </c>
       <c r="O52" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="53" spans="7:20" x14ac:dyDescent="0.45">
@@ -3449,7 +3593,7 @@
         <v>153</v>
       </c>
       <c r="O53" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="54" spans="7:20" x14ac:dyDescent="0.45">
@@ -3475,7 +3619,7 @@
         <v>155</v>
       </c>
       <c r="O54" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="55" spans="7:20" x14ac:dyDescent="0.45">
@@ -3483,10 +3627,10 @@
         <v>78</v>
       </c>
       <c r="H55" t="s">
-        <v>79</v>
+        <v>235</v>
       </c>
       <c r="I55" t="s">
-        <v>80</v>
+        <v>236</v>
       </c>
       <c r="J55" t="s">
         <v>158</v>
@@ -3495,13 +3639,13 @@
         <v>78</v>
       </c>
       <c r="M55" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="N55" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="O55" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="56" spans="7:20" x14ac:dyDescent="0.45">
@@ -3509,10 +3653,10 @@
         <v>78</v>
       </c>
       <c r="H56" t="s">
-        <v>235</v>
+        <v>79</v>
       </c>
       <c r="I56" t="s">
-        <v>236</v>
+        <v>80</v>
       </c>
       <c r="J56" t="s">
         <v>158</v>
@@ -3521,41 +3665,65 @@
         <v>78</v>
       </c>
       <c r="M56" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="N56" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="O56" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="57" spans="7:20" x14ac:dyDescent="0.45">
+      <c r="G57" t="s">
+        <v>78</v>
+      </c>
+      <c r="H57" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="57" spans="7:20" x14ac:dyDescent="0.45">
+      <c r="I57" t="s">
+        <v>238</v>
+      </c>
+      <c r="J57" t="s">
+        <v>158</v>
+      </c>
       <c r="L57" t="s">
         <v>78</v>
       </c>
       <c r="M57" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="N57" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="O57" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="58" spans="7:20" x14ac:dyDescent="0.45">
+      <c r="G58" t="s">
+        <v>78</v>
+      </c>
+      <c r="H58" t="s">
+        <v>140</v>
+      </c>
+      <c r="I58" t="s">
+        <v>141</v>
+      </c>
+      <c r="J58" t="s">
+        <v>158</v>
+      </c>
       <c r="L58" t="s">
         <v>78</v>
       </c>
       <c r="M58" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
       <c r="N58" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="O58" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="59" spans="7:20" x14ac:dyDescent="0.45">
@@ -3563,13 +3731,13 @@
         <v>78</v>
       </c>
       <c r="M59" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="N59" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="O59" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="60" spans="7:20" x14ac:dyDescent="0.45">
@@ -3577,13 +3745,13 @@
         <v>78</v>
       </c>
       <c r="M60" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="N60" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="O60" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="61" spans="7:20" x14ac:dyDescent="0.45">
@@ -3591,13 +3759,13 @@
         <v>78</v>
       </c>
       <c r="M61" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="N61" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="O61" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="62" spans="7:20" x14ac:dyDescent="0.45">
@@ -3605,13 +3773,13 @@
         <v>78</v>
       </c>
       <c r="M62" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="N62" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="O62" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="63" spans="7:20" x14ac:dyDescent="0.45">
@@ -3619,13 +3787,13 @@
         <v>78</v>
       </c>
       <c r="M63" t="s">
-        <v>260</v>
+        <v>171</v>
       </c>
       <c r="N63" t="s">
-        <v>261</v>
+        <v>172</v>
       </c>
       <c r="O63" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="64" spans="7:20" x14ac:dyDescent="0.45">
@@ -3639,7 +3807,7 @@
         <v>263</v>
       </c>
       <c r="O64" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="65" spans="12:15" x14ac:dyDescent="0.45">
@@ -3653,7 +3821,7 @@
         <v>265</v>
       </c>
       <c r="O65" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="66" spans="12:15" x14ac:dyDescent="0.45">
@@ -3667,7 +3835,7 @@
         <v>267</v>
       </c>
       <c r="O66" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="67" spans="12:15" x14ac:dyDescent="0.45">
@@ -3681,7 +3849,7 @@
         <v>269</v>
       </c>
       <c r="O67" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="68" spans="12:15" x14ac:dyDescent="0.45">
@@ -3689,13 +3857,13 @@
         <v>78</v>
       </c>
       <c r="M68" t="s">
-        <v>167</v>
+        <v>270</v>
       </c>
       <c r="N68" t="s">
-        <v>168</v>
+        <v>271</v>
       </c>
       <c r="O68" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="69" spans="12:15" x14ac:dyDescent="0.45">
@@ -3703,13 +3871,13 @@
         <v>78</v>
       </c>
       <c r="M69" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="N69" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="O69" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="70" spans="12:15" x14ac:dyDescent="0.45">
@@ -3717,13 +3885,13 @@
         <v>78</v>
       </c>
       <c r="M70" t="s">
-        <v>156</v>
+        <v>187</v>
       </c>
       <c r="N70" t="s">
-        <v>157</v>
+        <v>188</v>
       </c>
       <c r="O70" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="71" spans="12:15" x14ac:dyDescent="0.45">
@@ -3731,13 +3899,13 @@
         <v>78</v>
       </c>
       <c r="M71" t="s">
-        <v>159</v>
+        <v>274</v>
       </c>
       <c r="N71" t="s">
-        <v>160</v>
+        <v>275</v>
       </c>
       <c r="O71" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="72" spans="12:15" x14ac:dyDescent="0.45">
@@ -3745,13 +3913,13 @@
         <v>78</v>
       </c>
       <c r="M72" t="s">
-        <v>161</v>
+        <v>276</v>
       </c>
       <c r="N72" t="s">
-        <v>162</v>
+        <v>277</v>
       </c>
       <c r="O72" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="73" spans="12:15" x14ac:dyDescent="0.45">
@@ -3759,13 +3927,13 @@
         <v>78</v>
       </c>
       <c r="M73" t="s">
-        <v>163</v>
+        <v>278</v>
       </c>
       <c r="N73" t="s">
-        <v>164</v>
+        <v>279</v>
       </c>
       <c r="O73" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="74" spans="12:15" x14ac:dyDescent="0.45">
@@ -3773,13 +3941,13 @@
         <v>78</v>
       </c>
       <c r="M74" t="s">
-        <v>165</v>
+        <v>280</v>
       </c>
       <c r="N74" t="s">
-        <v>166</v>
+        <v>281</v>
       </c>
       <c r="O74" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="75" spans="12:15" x14ac:dyDescent="0.45">
@@ -3787,13 +3955,13 @@
         <v>78</v>
       </c>
       <c r="M75" t="s">
-        <v>169</v>
+        <v>282</v>
       </c>
       <c r="N75" t="s">
-        <v>170</v>
+        <v>283</v>
       </c>
       <c r="O75" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="76" spans="12:15" x14ac:dyDescent="0.45">
@@ -3801,13 +3969,13 @@
         <v>78</v>
       </c>
       <c r="M76" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="N76" t="s">
-        <v>172</v>
+        <v>285</v>
       </c>
       <c r="O76" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="77" spans="12:15" x14ac:dyDescent="0.45">
@@ -3815,13 +3983,13 @@
         <v>78</v>
       </c>
       <c r="M77" t="s">
-        <v>173</v>
+        <v>286</v>
       </c>
       <c r="N77" t="s">
-        <v>174</v>
+        <v>287</v>
       </c>
       <c r="O77" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="78" spans="12:15" x14ac:dyDescent="0.45">
@@ -3829,13 +3997,13 @@
         <v>78</v>
       </c>
       <c r="M78" t="s">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="N78" t="s">
-        <v>176</v>
+        <v>162</v>
       </c>
       <c r="O78" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="79" spans="12:15" x14ac:dyDescent="0.45">
@@ -3843,13 +4011,13 @@
         <v>78</v>
       </c>
       <c r="M79" t="s">
-        <v>177</v>
+        <v>288</v>
       </c>
       <c r="N79" t="s">
-        <v>178</v>
+        <v>289</v>
       </c>
       <c r="O79" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="80" spans="12:15" x14ac:dyDescent="0.45">
@@ -3857,13 +4025,13 @@
         <v>78</v>
       </c>
       <c r="M80" t="s">
-        <v>179</v>
+        <v>290</v>
       </c>
       <c r="N80" t="s">
-        <v>180</v>
+        <v>291</v>
       </c>
       <c r="O80" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="81" spans="12:15" x14ac:dyDescent="0.45">
@@ -3871,13 +4039,13 @@
         <v>78</v>
       </c>
       <c r="M81" t="s">
-        <v>181</v>
+        <v>201</v>
       </c>
       <c r="N81" t="s">
-        <v>182</v>
+        <v>202</v>
       </c>
       <c r="O81" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="82" spans="12:15" x14ac:dyDescent="0.45">
@@ -3885,13 +4053,13 @@
         <v>78</v>
       </c>
       <c r="M82" t="s">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="N82" t="s">
-        <v>186</v>
+        <v>222</v>
       </c>
       <c r="O82" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="83" spans="12:15" x14ac:dyDescent="0.45">
@@ -3899,13 +4067,13 @@
         <v>78</v>
       </c>
       <c r="M83" t="s">
-        <v>187</v>
+        <v>292</v>
       </c>
       <c r="N83" t="s">
-        <v>188</v>
+        <v>293</v>
       </c>
       <c r="O83" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="84" spans="12:15" x14ac:dyDescent="0.45">
@@ -3913,13 +4081,13 @@
         <v>78</v>
       </c>
       <c r="M84" t="s">
-        <v>189</v>
+        <v>294</v>
       </c>
       <c r="N84" t="s">
-        <v>190</v>
+        <v>295</v>
       </c>
       <c r="O84" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="85" spans="12:15" x14ac:dyDescent="0.45">
@@ -3927,13 +4095,13 @@
         <v>78</v>
       </c>
       <c r="M85" t="s">
-        <v>191</v>
+        <v>296</v>
       </c>
       <c r="N85" t="s">
-        <v>192</v>
+        <v>297</v>
       </c>
       <c r="O85" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="86" spans="12:15" x14ac:dyDescent="0.45">
@@ -3941,13 +4109,13 @@
         <v>78</v>
       </c>
       <c r="M86" t="s">
-        <v>193</v>
+        <v>298</v>
       </c>
       <c r="N86" t="s">
-        <v>194</v>
+        <v>299</v>
       </c>
       <c r="O86" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="87" spans="12:15" x14ac:dyDescent="0.45">
@@ -3955,13 +4123,13 @@
         <v>78</v>
       </c>
       <c r="M87" t="s">
-        <v>195</v>
+        <v>300</v>
       </c>
       <c r="N87" t="s">
-        <v>196</v>
+        <v>301</v>
       </c>
       <c r="O87" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="88" spans="12:15" x14ac:dyDescent="0.45">
@@ -3969,13 +4137,13 @@
         <v>78</v>
       </c>
       <c r="M88" t="s">
-        <v>197</v>
+        <v>302</v>
       </c>
       <c r="N88" t="s">
-        <v>198</v>
+        <v>303</v>
       </c>
       <c r="O88" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="89" spans="12:15" x14ac:dyDescent="0.45">
@@ -3983,13 +4151,13 @@
         <v>78</v>
       </c>
       <c r="M89" t="s">
-        <v>199</v>
+        <v>304</v>
       </c>
       <c r="N89" t="s">
-        <v>200</v>
+        <v>305</v>
       </c>
       <c r="O89" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="90" spans="12:15" x14ac:dyDescent="0.45">
@@ -3997,13 +4165,13 @@
         <v>78</v>
       </c>
       <c r="M90" t="s">
-        <v>201</v>
+        <v>306</v>
       </c>
       <c r="N90" t="s">
-        <v>202</v>
+        <v>307</v>
       </c>
       <c r="O90" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="91" spans="12:15" x14ac:dyDescent="0.45">
@@ -4011,13 +4179,13 @@
         <v>78</v>
       </c>
       <c r="M91" t="s">
-        <v>207</v>
+        <v>308</v>
       </c>
       <c r="N91" t="s">
-        <v>208</v>
+        <v>309</v>
       </c>
       <c r="O91" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="92" spans="12:15" x14ac:dyDescent="0.45">
@@ -4025,13 +4193,13 @@
         <v>78</v>
       </c>
       <c r="M92" t="s">
-        <v>209</v>
+        <v>310</v>
       </c>
       <c r="N92" t="s">
-        <v>210</v>
+        <v>311</v>
       </c>
       <c r="O92" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="93" spans="12:15" x14ac:dyDescent="0.45">
@@ -4039,13 +4207,13 @@
         <v>78</v>
       </c>
       <c r="M93" t="s">
-        <v>211</v>
+        <v>169</v>
       </c>
       <c r="N93" t="s">
-        <v>212</v>
+        <v>170</v>
       </c>
       <c r="O93" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="94" spans="12:15" x14ac:dyDescent="0.45">
@@ -4053,13 +4221,13 @@
         <v>78</v>
       </c>
       <c r="M94" t="s">
-        <v>213</v>
+        <v>312</v>
       </c>
       <c r="N94" t="s">
-        <v>214</v>
+        <v>313</v>
       </c>
       <c r="O94" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="95" spans="12:15" x14ac:dyDescent="0.45">
@@ -4067,13 +4235,13 @@
         <v>78</v>
       </c>
       <c r="M95" t="s">
-        <v>215</v>
+        <v>314</v>
       </c>
       <c r="N95" t="s">
-        <v>216</v>
+        <v>315</v>
       </c>
       <c r="O95" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="96" spans="12:15" x14ac:dyDescent="0.45">
@@ -4081,13 +4249,13 @@
         <v>78</v>
       </c>
       <c r="M96" t="s">
-        <v>217</v>
+        <v>316</v>
       </c>
       <c r="N96" t="s">
-        <v>218</v>
+        <v>317</v>
       </c>
       <c r="O96" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="97" spans="12:15" x14ac:dyDescent="0.45">
@@ -4095,13 +4263,13 @@
         <v>78</v>
       </c>
       <c r="M97" t="s">
-        <v>219</v>
+        <v>318</v>
       </c>
       <c r="N97" t="s">
-        <v>220</v>
+        <v>319</v>
       </c>
       <c r="O97" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="98" spans="12:15" x14ac:dyDescent="0.45">
@@ -4109,13 +4277,13 @@
         <v>78</v>
       </c>
       <c r="M98" t="s">
-        <v>221</v>
+        <v>320</v>
       </c>
       <c r="N98" t="s">
-        <v>222</v>
+        <v>321</v>
       </c>
       <c r="O98" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="99" spans="12:15" x14ac:dyDescent="0.45">
@@ -4123,13 +4291,13 @@
         <v>78</v>
       </c>
       <c r="M99" t="s">
-        <v>223</v>
+        <v>322</v>
       </c>
       <c r="N99" t="s">
-        <v>224</v>
+        <v>323</v>
       </c>
       <c r="O99" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="100" spans="12:15" x14ac:dyDescent="0.45">
@@ -4137,13 +4305,13 @@
         <v>78</v>
       </c>
       <c r="M100" t="s">
-        <v>225</v>
+        <v>324</v>
       </c>
       <c r="N100" t="s">
-        <v>226</v>
+        <v>325</v>
       </c>
       <c r="O100" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="101" spans="12:15" x14ac:dyDescent="0.45">
@@ -4151,13 +4319,13 @@
         <v>78</v>
       </c>
       <c r="M101" t="s">
-        <v>227</v>
+        <v>326</v>
       </c>
       <c r="N101" t="s">
-        <v>228</v>
+        <v>327</v>
       </c>
       <c r="O101" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="102" spans="12:15" x14ac:dyDescent="0.45">
@@ -4165,13 +4333,13 @@
         <v>78</v>
       </c>
       <c r="M102" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="N102" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="O102" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="103" spans="12:15" x14ac:dyDescent="0.45">
@@ -4179,13 +4347,13 @@
         <v>78</v>
       </c>
       <c r="M103" t="s">
-        <v>231</v>
+        <v>156</v>
       </c>
       <c r="N103" t="s">
-        <v>232</v>
+        <v>157</v>
       </c>
       <c r="O103" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="104" spans="12:15" x14ac:dyDescent="0.45">
@@ -4193,13 +4361,13 @@
         <v>78</v>
       </c>
       <c r="M104" t="s">
-        <v>233</v>
+        <v>159</v>
       </c>
       <c r="N104" t="s">
-        <v>234</v>
+        <v>160</v>
       </c>
       <c r="O104" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="105" spans="12:15" x14ac:dyDescent="0.45">
@@ -4207,13 +4375,13 @@
         <v>78</v>
       </c>
       <c r="M105" t="s">
-        <v>235</v>
+        <v>163</v>
       </c>
       <c r="N105" t="s">
-        <v>236</v>
+        <v>164</v>
       </c>
       <c r="O105" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="106" spans="12:15" x14ac:dyDescent="0.45">
@@ -4221,13 +4389,13 @@
         <v>78</v>
       </c>
       <c r="M106" t="s">
-        <v>272</v>
+        <v>165</v>
       </c>
       <c r="N106" t="s">
-        <v>273</v>
+        <v>166</v>
       </c>
       <c r="O106" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="107" spans="12:15" x14ac:dyDescent="0.45">
@@ -4235,13 +4403,405 @@
         <v>78</v>
       </c>
       <c r="M107" t="s">
-        <v>274</v>
+        <v>167</v>
       </c>
       <c r="N107" t="s">
-        <v>275</v>
+        <v>168</v>
       </c>
       <c r="O107" t="s">
-        <v>237</v>
+        <v>239</v>
+      </c>
+    </row>
+    <row r="108" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L108" t="s">
+        <v>78</v>
+      </c>
+      <c r="M108" t="s">
+        <v>173</v>
+      </c>
+      <c r="N108" t="s">
+        <v>174</v>
+      </c>
+      <c r="O108" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="109" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L109" t="s">
+        <v>78</v>
+      </c>
+      <c r="M109" t="s">
+        <v>175</v>
+      </c>
+      <c r="N109" t="s">
+        <v>176</v>
+      </c>
+      <c r="O109" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="110" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L110" t="s">
+        <v>78</v>
+      </c>
+      <c r="M110" t="s">
+        <v>177</v>
+      </c>
+      <c r="N110" t="s">
+        <v>178</v>
+      </c>
+      <c r="O110" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="111" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L111" t="s">
+        <v>78</v>
+      </c>
+      <c r="M111" t="s">
+        <v>179</v>
+      </c>
+      <c r="N111" t="s">
+        <v>180</v>
+      </c>
+      <c r="O111" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="112" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L112" t="s">
+        <v>78</v>
+      </c>
+      <c r="M112" t="s">
+        <v>183</v>
+      </c>
+      <c r="N112" t="s">
+        <v>184</v>
+      </c>
+      <c r="O112" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="113" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L113" t="s">
+        <v>78</v>
+      </c>
+      <c r="M113" t="s">
+        <v>189</v>
+      </c>
+      <c r="N113" t="s">
+        <v>190</v>
+      </c>
+      <c r="O113" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="114" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L114" t="s">
+        <v>78</v>
+      </c>
+      <c r="M114" t="s">
+        <v>191</v>
+      </c>
+      <c r="N114" t="s">
+        <v>192</v>
+      </c>
+      <c r="O114" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="115" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L115" t="s">
+        <v>78</v>
+      </c>
+      <c r="M115" t="s">
+        <v>193</v>
+      </c>
+      <c r="N115" t="s">
+        <v>194</v>
+      </c>
+      <c r="O115" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="116" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L116" t="s">
+        <v>78</v>
+      </c>
+      <c r="M116" t="s">
+        <v>195</v>
+      </c>
+      <c r="N116" t="s">
+        <v>196</v>
+      </c>
+      <c r="O116" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="117" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L117" t="s">
+        <v>78</v>
+      </c>
+      <c r="M117" t="s">
+        <v>197</v>
+      </c>
+      <c r="N117" t="s">
+        <v>198</v>
+      </c>
+      <c r="O117" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="118" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L118" t="s">
+        <v>78</v>
+      </c>
+      <c r="M118" t="s">
+        <v>199</v>
+      </c>
+      <c r="N118" t="s">
+        <v>200</v>
+      </c>
+      <c r="O118" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="119" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L119" t="s">
+        <v>78</v>
+      </c>
+      <c r="M119" t="s">
+        <v>203</v>
+      </c>
+      <c r="N119" t="s">
+        <v>204</v>
+      </c>
+      <c r="O119" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="120" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L120" t="s">
+        <v>78</v>
+      </c>
+      <c r="M120" t="s">
+        <v>207</v>
+      </c>
+      <c r="N120" t="s">
+        <v>208</v>
+      </c>
+      <c r="O120" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="121" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L121" t="s">
+        <v>78</v>
+      </c>
+      <c r="M121" t="s">
+        <v>209</v>
+      </c>
+      <c r="N121" t="s">
+        <v>210</v>
+      </c>
+      <c r="O121" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="122" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L122" t="s">
+        <v>78</v>
+      </c>
+      <c r="M122" t="s">
+        <v>211</v>
+      </c>
+      <c r="N122" t="s">
+        <v>212</v>
+      </c>
+      <c r="O122" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="123" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L123" t="s">
+        <v>78</v>
+      </c>
+      <c r="M123" t="s">
+        <v>213</v>
+      </c>
+      <c r="N123" t="s">
+        <v>214</v>
+      </c>
+      <c r="O123" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="124" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L124" t="s">
+        <v>78</v>
+      </c>
+      <c r="M124" t="s">
+        <v>215</v>
+      </c>
+      <c r="N124" t="s">
+        <v>216</v>
+      </c>
+      <c r="O124" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="125" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L125" t="s">
+        <v>78</v>
+      </c>
+      <c r="M125" t="s">
+        <v>217</v>
+      </c>
+      <c r="N125" t="s">
+        <v>218</v>
+      </c>
+      <c r="O125" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="126" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L126" t="s">
+        <v>78</v>
+      </c>
+      <c r="M126" t="s">
+        <v>219</v>
+      </c>
+      <c r="N126" t="s">
+        <v>220</v>
+      </c>
+      <c r="O126" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="127" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L127" t="s">
+        <v>78</v>
+      </c>
+      <c r="M127" t="s">
+        <v>223</v>
+      </c>
+      <c r="N127" t="s">
+        <v>224</v>
+      </c>
+      <c r="O127" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="128" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L128" t="s">
+        <v>78</v>
+      </c>
+      <c r="M128" t="s">
+        <v>225</v>
+      </c>
+      <c r="N128" t="s">
+        <v>226</v>
+      </c>
+      <c r="O128" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="129" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L129" t="s">
+        <v>78</v>
+      </c>
+      <c r="M129" t="s">
+        <v>227</v>
+      </c>
+      <c r="N129" t="s">
+        <v>228</v>
+      </c>
+      <c r="O129" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="130" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L130" t="s">
+        <v>78</v>
+      </c>
+      <c r="M130" t="s">
+        <v>229</v>
+      </c>
+      <c r="N130" t="s">
+        <v>230</v>
+      </c>
+      <c r="O130" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="131" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L131" t="s">
+        <v>78</v>
+      </c>
+      <c r="M131" t="s">
+        <v>231</v>
+      </c>
+      <c r="N131" t="s">
+        <v>232</v>
+      </c>
+      <c r="O131" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="132" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L132" t="s">
+        <v>78</v>
+      </c>
+      <c r="M132" t="s">
+        <v>233</v>
+      </c>
+      <c r="N132" t="s">
+        <v>234</v>
+      </c>
+      <c r="O132" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="133" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L133" t="s">
+        <v>78</v>
+      </c>
+      <c r="M133" t="s">
+        <v>235</v>
+      </c>
+      <c r="N133" t="s">
+        <v>236</v>
+      </c>
+      <c r="O133" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="134" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L134" t="s">
+        <v>78</v>
+      </c>
+      <c r="M134" t="s">
+        <v>328</v>
+      </c>
+      <c r="N134" t="s">
+        <v>329</v>
+      </c>
+      <c r="O134" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="135" spans="12:15" x14ac:dyDescent="0.45">
+      <c r="L135" t="s">
+        <v>78</v>
+      </c>
+      <c r="M135" t="s">
+        <v>330</v>
+      </c>
+      <c r="N135" t="s">
+        <v>331</v>
+      </c>
+      <c r="O135" t="s">
+        <v>239</v>
       </c>
     </row>
   </sheetData>

</xml_diff>